<commit_message>
etsy: casamento sem cara de IA (status em palavras, textos simples, fotos novas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/wedding/Wedding-Budget-Planner.xlsx
+++ b/etsy/wedding/Wedding-Budget-Planner.xlsx
@@ -114,7 +114,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -123,8 +123,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F4EF"/>
-        <bgColor rgb="00F6F4EF"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,12 +137,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F6F78"/>
         <bgColor rgb="001F6F78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -186,23 +180,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </bottom>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -210,10 +204,10 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -221,13 +215,13 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -242,32 +236,34 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="10" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -275,13 +271,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -292,6 +288,14 @@
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D8F0DC"/>
+          <bgColor rgb="00D8F0DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -316,14 +320,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00D8F0DC"/>
-          <bgColor rgb="00D8F0DC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="00FFE2B8"/>
           <bgColor rgb="00FFE2B8"/>
         </patternFill>
@@ -332,8 +328,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00E6E2DA"/>
-          <bgColor rgb="00E6E2DA"/>
+          <fgColor rgb="00E4E8E8"/>
+          <bgColor rgb="00E4E8E8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -727,7 +723,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Our wedding at a glance</t>
+          <t>Wedding dashboard</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -899,24 +895,24 @@
         </is>
       </c>
       <c r="C10" s="14">
-        <f>COUNTIFS(Guests!$B$6:$B$305,"&lt;&gt;")+COUNTIFS(Guests!$B$6:$B$305,"&lt;&gt;",Guests!$E$6:$E$305,TRUE)</f>
+        <f>COUNTIFS(Guests!$B$6:$B$305,"&lt;&gt;")+COUNTIFS(Guests!$B$6:$B$305,"&lt;&gt;",Guests!$E$6:$E$305,"Yes")</f>
         <v/>
       </c>
       <c r="D10" s="14">
-        <f>COUNTIFS(Guests!$D$6:$D$305,"Yes")+COUNTIFS(Guests!$D$6:$D$305,"Yes",Guests!$E$6:$E$305,TRUE)</f>
+        <f>COUNTIFS(Guests!$D$6:$D$305,"Yes")+COUNTIFS(Guests!$D$6:$D$305,"Yes",Guests!$E$6:$E$305,"Yes")</f>
         <v/>
       </c>
       <c r="E10" s="14">
-        <f>COUNTIFS(Guests!$D$6:$D$305,"Pending")+COUNTIFS(Guests!$D$6:$D$305,"Pending",Guests!$E$6:$E$305,TRUE)</f>
+        <f>COUNTIFS(Guests!$D$6:$D$305,"Pending")+COUNTIFS(Guests!$D$6:$D$305,"Pending",Guests!$E$6:$E$305,"Yes")</f>
         <v/>
       </c>
       <c r="F10" s="14">
-        <f>COUNTIFS(Guests!$D$6:$D$305,"No")+COUNTIFS(Guests!$D$6:$D$305,"No",Guests!$E$6:$E$305,TRUE)</f>
+        <f>COUNTIFS(Guests!$D$6:$D$305,"No")+COUNTIFS(Guests!$D$6:$D$305,"No",Guests!$E$6:$E$305,"Yes")</f>
         <v/>
       </c>
       <c r="G10" s="1" t="n"/>
       <c r="H10" s="15">
-        <f>COUNTIFS(Vendors!$H$6:$H$105,"⚠*")&amp;" payment(s) overdue"</f>
+        <f>IF(COUNTIFS(Vendors!$H$6:$H$105,"Overdue*")=0,"No overdue payments",IF(COUNTIFS(Vendors!$H$6:$H$105,"Overdue*")=1,"1 payment is overdue",COUNTIFS(Vendors!$H$6:$H$105,"Overdue*")&amp;" payments are overdue"))</f>
         <v/>
       </c>
       <c r="I10" s="1" t="n"/>
@@ -946,7 +942,7 @@
       </c>
       <c r="G11" s="1" t="n"/>
       <c r="H11" s="17">
-        <f>COUNTIFS(Vendors!$H$6:$H$105,"Due in*")&amp;" payment(s) due in the next 14 days: "&amp;FIXED(SUMIFS(Vendors!$G$6:$G$105,Vendors!$H$6:$H$105,"Due in*"),2)</f>
+        <f>IF((COUNTIFS(Vendors!$H$6:$H$105,"Due in*")+COUNTIFS(Vendors!$H$6:$H$105,"Due today"))=0,"Nothing due in the next 14 days",IF((COUNTIFS(Vendors!$H$6:$H$105,"Due in*")+COUNTIFS(Vendors!$H$6:$H$105,"Due today"))=1,"1 payment",(COUNTIFS(Vendors!$H$6:$H$105,"Due in*")+COUNTIFS(Vendors!$H$6:$H$105,"Due today"))&amp;" payments")&amp;" due in the next 14 days: "&amp;FIXED((SUMIFS(Vendors!$G$6:$G$105,Vendors!$H$6:$H$105,"Due in*")+SUMIFS(Vendors!$G$6:$G$105,Vendors!$H$6:$H$105,"Due today")),2))</f>
         <v/>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -960,7 +956,7 @@
       <c r="F12" s="1" t="n"/>
       <c r="G12" s="1" t="n"/>
       <c r="H12" s="18">
-        <f>COUNTIFS(Guests!$D$6:$D$305,"Pending")&amp;" guest(s) still to answer"</f>
+        <f>IF(COUNTIFS(Guests!$D$6:$D$305,"Pending")=0,"Every guest has answered",IF(COUNTIFS(Guests!$D$6:$D$305,"Pending")=1,"1 guest has not answered yet",COUNTIFS(Guests!$D$6:$D$305,"Pending")&amp;" guests have not answered yet"))</f>
         <v/>
       </c>
       <c r="I12" s="1" t="n"/>
@@ -1854,8 +1850,28 @@
       <c r="I79" s="1" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>LEFT(H10,2)="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>LEFT(H11,7)="Nothing"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>LEFT(H12,5)="Every"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>LEFT(H13,4)="Over"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D15:D25">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="5" dxfId="1">
       <formula>$D15&gt;$C15</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3049,12 +3065,12 @@
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <conditionalFormatting sqref="C17">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="1">
       <formula>$C$17&lt;&gt;100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:E16">
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="2">
       <formula>$E6&gt;$D6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3199,7 +3215,7 @@
         <v/>
       </c>
       <c r="H6" s="33">
-        <f>IF(B6="","",IF(G6&lt;=0,"✓ Paid in full",IF(F6="","Balance, no date yet",IF(F6&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F6)&amp;" day(s)",IF(F6-TODAY()&lt;=14,"Due in "&amp;(F6-TODAY())&amp;" day(s)","Due "&amp;(F6-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B6="","",IF(G6&lt;=0,"Paid in full",IF(F6="","Balance due, no date set",IF(F6&lt;TODAY(),"Overdue by "&amp;TODAY()-F6&amp;IF(TODAY()-F6=1," day"," days"),IF(F6=TODAY(),"Due today",IF(F6-TODAY()&lt;=14,"Due in "&amp;F6-TODAY()&amp;IF(F6-TODAY()=1," day"," days"),"Next payment in "&amp;F6-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I6" s="1" t="n"/>
@@ -3230,7 +3246,7 @@
         <v/>
       </c>
       <c r="H7" s="33">
-        <f>IF(B7="","",IF(G7&lt;=0,"✓ Paid in full",IF(F7="","Balance, no date yet",IF(F7&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F7)&amp;" day(s)",IF(F7-TODAY()&lt;=14,"Due in "&amp;(F7-TODAY())&amp;" day(s)","Due "&amp;(F7-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B7="","",IF(G7&lt;=0,"Paid in full",IF(F7="","Balance due, no date set",IF(F7&lt;TODAY(),"Overdue by "&amp;TODAY()-F7&amp;IF(TODAY()-F7=1," day"," days"),IF(F7=TODAY(),"Due today",IF(F7-TODAY()&lt;=14,"Due in "&amp;F7-TODAY()&amp;IF(F7-TODAY()=1," day"," days"),"Next payment in "&amp;F7-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I7" s="1" t="n"/>
@@ -3261,7 +3277,7 @@
         <v/>
       </c>
       <c r="H8" s="33">
-        <f>IF(B8="","",IF(G8&lt;=0,"✓ Paid in full",IF(F8="","Balance, no date yet",IF(F8&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F8)&amp;" day(s)",IF(F8-TODAY()&lt;=14,"Due in "&amp;(F8-TODAY())&amp;" day(s)","Due "&amp;(F8-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B8="","",IF(G8&lt;=0,"Paid in full",IF(F8="","Balance due, no date set",IF(F8&lt;TODAY(),"Overdue by "&amp;TODAY()-F8&amp;IF(TODAY()-F8=1," day"," days"),IF(F8=TODAY(),"Due today",IF(F8-TODAY()&lt;=14,"Due in "&amp;F8-TODAY()&amp;IF(F8-TODAY()=1," day"," days"),"Next payment in "&amp;F8-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I8" s="1" t="n"/>
@@ -3290,7 +3306,7 @@
         <v/>
       </c>
       <c r="H9" s="33">
-        <f>IF(B9="","",IF(G9&lt;=0,"✓ Paid in full",IF(F9="","Balance, no date yet",IF(F9&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F9)&amp;" day(s)",IF(F9-TODAY()&lt;=14,"Due in "&amp;(F9-TODAY())&amp;" day(s)","Due "&amp;(F9-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B9="","",IF(G9&lt;=0,"Paid in full",IF(F9="","Balance due, no date set",IF(F9&lt;TODAY(),"Overdue by "&amp;TODAY()-F9&amp;IF(TODAY()-F9=1," day"," days"),IF(F9=TODAY(),"Due today",IF(F9-TODAY()&lt;=14,"Due in "&amp;F9-TODAY()&amp;IF(F9-TODAY()=1," day"," days"),"Next payment in "&amp;F9-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I9" s="1" t="n"/>
@@ -3321,7 +3337,7 @@
         <v/>
       </c>
       <c r="H10" s="33">
-        <f>IF(B10="","",IF(G10&lt;=0,"✓ Paid in full",IF(F10="","Balance, no date yet",IF(F10&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F10)&amp;" day(s)",IF(F10-TODAY()&lt;=14,"Due in "&amp;(F10-TODAY())&amp;" day(s)","Due "&amp;(F10-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B10="","",IF(G10&lt;=0,"Paid in full",IF(F10="","Balance due, no date set",IF(F10&lt;TODAY(),"Overdue by "&amp;TODAY()-F10&amp;IF(TODAY()-F10=1," day"," days"),IF(F10=TODAY(),"Due today",IF(F10-TODAY()&lt;=14,"Due in "&amp;F10-TODAY()&amp;IF(F10-TODAY()=1," day"," days"),"Next payment in "&amp;F10-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I10" s="1" t="n"/>
@@ -3352,7 +3368,7 @@
         <v/>
       </c>
       <c r="H11" s="33">
-        <f>IF(B11="","",IF(G11&lt;=0,"✓ Paid in full",IF(F11="","Balance, no date yet",IF(F11&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F11)&amp;" day(s)",IF(F11-TODAY()&lt;=14,"Due in "&amp;(F11-TODAY())&amp;" day(s)","Due "&amp;(F11-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B11="","",IF(G11&lt;=0,"Paid in full",IF(F11="","Balance due, no date set",IF(F11&lt;TODAY(),"Overdue by "&amp;TODAY()-F11&amp;IF(TODAY()-F11=1," day"," days"),IF(F11=TODAY(),"Due today",IF(F11-TODAY()&lt;=14,"Due in "&amp;F11-TODAY()&amp;IF(F11-TODAY()=1," day"," days"),"Next payment in "&amp;F11-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -3381,7 +3397,7 @@
         <v/>
       </c>
       <c r="H12" s="33">
-        <f>IF(B12="","",IF(G12&lt;=0,"✓ Paid in full",IF(F12="","Balance, no date yet",IF(F12&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F12)&amp;" day(s)",IF(F12-TODAY()&lt;=14,"Due in "&amp;(F12-TODAY())&amp;" day(s)","Due "&amp;(F12-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B12="","",IF(G12&lt;=0,"Paid in full",IF(F12="","Balance due, no date set",IF(F12&lt;TODAY(),"Overdue by "&amp;TODAY()-F12&amp;IF(TODAY()-F12=1," day"," days"),IF(F12=TODAY(),"Due today",IF(F12-TODAY()&lt;=14,"Due in "&amp;F12-TODAY()&amp;IF(F12-TODAY()=1," day"," days"),"Next payment in "&amp;F12-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I12" s="1" t="n"/>
@@ -3412,7 +3428,7 @@
         <v/>
       </c>
       <c r="H13" s="33">
-        <f>IF(B13="","",IF(G13&lt;=0,"✓ Paid in full",IF(F13="","Balance, no date yet",IF(F13&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F13)&amp;" day(s)",IF(F13-TODAY()&lt;=14,"Due in "&amp;(F13-TODAY())&amp;" day(s)","Due "&amp;(F13-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B13="","",IF(G13&lt;=0,"Paid in full",IF(F13="","Balance due, no date set",IF(F13&lt;TODAY(),"Overdue by "&amp;TODAY()-F13&amp;IF(TODAY()-F13=1," day"," days"),IF(F13=TODAY(),"Due today",IF(F13-TODAY()&lt;=14,"Due in "&amp;F13-TODAY()&amp;IF(F13-TODAY()=1," day"," days"),"Next payment in "&amp;F13-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -3429,7 +3445,7 @@
         <v/>
       </c>
       <c r="H14" s="33">
-        <f>IF(B14="","",IF(G14&lt;=0,"✓ Paid in full",IF(F14="","Balance, no date yet",IF(F14&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F14)&amp;" day(s)",IF(F14-TODAY()&lt;=14,"Due in "&amp;(F14-TODAY())&amp;" day(s)","Due "&amp;(F14-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B14="","",IF(G14&lt;=0,"Paid in full",IF(F14="","Balance due, no date set",IF(F14&lt;TODAY(),"Overdue by "&amp;TODAY()-F14&amp;IF(TODAY()-F14=1," day"," days"),IF(F14=TODAY(),"Due today",IF(F14-TODAY()&lt;=14,"Due in "&amp;F14-TODAY()&amp;IF(F14-TODAY()=1," day"," days"),"Next payment in "&amp;F14-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I14" s="1" t="n"/>
@@ -3446,7 +3462,7 @@
         <v/>
       </c>
       <c r="H15" s="33">
-        <f>IF(B15="","",IF(G15&lt;=0,"✓ Paid in full",IF(F15="","Balance, no date yet",IF(F15&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F15)&amp;" day(s)",IF(F15-TODAY()&lt;=14,"Due in "&amp;(F15-TODAY())&amp;" day(s)","Due "&amp;(F15-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B15="","",IF(G15&lt;=0,"Paid in full",IF(F15="","Balance due, no date set",IF(F15&lt;TODAY(),"Overdue by "&amp;TODAY()-F15&amp;IF(TODAY()-F15=1," day"," days"),IF(F15=TODAY(),"Due today",IF(F15-TODAY()&lt;=14,"Due in "&amp;F15-TODAY()&amp;IF(F15-TODAY()=1," day"," days"),"Next payment in "&amp;F15-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I15" s="1" t="n"/>
@@ -3463,7 +3479,7 @@
         <v/>
       </c>
       <c r="H16" s="33">
-        <f>IF(B16="","",IF(G16&lt;=0,"✓ Paid in full",IF(F16="","Balance, no date yet",IF(F16&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F16)&amp;" day(s)",IF(F16-TODAY()&lt;=14,"Due in "&amp;(F16-TODAY())&amp;" day(s)","Due "&amp;(F16-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B16="","",IF(G16&lt;=0,"Paid in full",IF(F16="","Balance due, no date set",IF(F16&lt;TODAY(),"Overdue by "&amp;TODAY()-F16&amp;IF(TODAY()-F16=1," day"," days"),IF(F16=TODAY(),"Due today",IF(F16-TODAY()&lt;=14,"Due in "&amp;F16-TODAY()&amp;IF(F16-TODAY()=1," day"," days"),"Next payment in "&amp;F16-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I16" s="1" t="n"/>
@@ -3480,7 +3496,7 @@
         <v/>
       </c>
       <c r="H17" s="33">
-        <f>IF(B17="","",IF(G17&lt;=0,"✓ Paid in full",IF(F17="","Balance, no date yet",IF(F17&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F17)&amp;" day(s)",IF(F17-TODAY()&lt;=14,"Due in "&amp;(F17-TODAY())&amp;" day(s)","Due "&amp;(F17-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B17="","",IF(G17&lt;=0,"Paid in full",IF(F17="","Balance due, no date set",IF(F17&lt;TODAY(),"Overdue by "&amp;TODAY()-F17&amp;IF(TODAY()-F17=1," day"," days"),IF(F17=TODAY(),"Due today",IF(F17-TODAY()&lt;=14,"Due in "&amp;F17-TODAY()&amp;IF(F17-TODAY()=1," day"," days"),"Next payment in "&amp;F17-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I17" s="1" t="n"/>
@@ -3497,7 +3513,7 @@
         <v/>
       </c>
       <c r="H18" s="33">
-        <f>IF(B18="","",IF(G18&lt;=0,"✓ Paid in full",IF(F18="","Balance, no date yet",IF(F18&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F18)&amp;" day(s)",IF(F18-TODAY()&lt;=14,"Due in "&amp;(F18-TODAY())&amp;" day(s)","Due "&amp;(F18-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B18="","",IF(G18&lt;=0,"Paid in full",IF(F18="","Balance due, no date set",IF(F18&lt;TODAY(),"Overdue by "&amp;TODAY()-F18&amp;IF(TODAY()-F18=1," day"," days"),IF(F18=TODAY(),"Due today",IF(F18-TODAY()&lt;=14,"Due in "&amp;F18-TODAY()&amp;IF(F18-TODAY()=1," day"," days"),"Next payment in "&amp;F18-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I18" s="1" t="n"/>
@@ -3514,7 +3530,7 @@
         <v/>
       </c>
       <c r="H19" s="33">
-        <f>IF(B19="","",IF(G19&lt;=0,"✓ Paid in full",IF(F19="","Balance, no date yet",IF(F19&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F19)&amp;" day(s)",IF(F19-TODAY()&lt;=14,"Due in "&amp;(F19-TODAY())&amp;" day(s)","Due "&amp;(F19-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B19="","",IF(G19&lt;=0,"Paid in full",IF(F19="","Balance due, no date set",IF(F19&lt;TODAY(),"Overdue by "&amp;TODAY()-F19&amp;IF(TODAY()-F19=1," day"," days"),IF(F19=TODAY(),"Due today",IF(F19-TODAY()&lt;=14,"Due in "&amp;F19-TODAY()&amp;IF(F19-TODAY()=1," day"," days"),"Next payment in "&amp;F19-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I19" s="1" t="n"/>
@@ -3531,7 +3547,7 @@
         <v/>
       </c>
       <c r="H20" s="33">
-        <f>IF(B20="","",IF(G20&lt;=0,"✓ Paid in full",IF(F20="","Balance, no date yet",IF(F20&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F20)&amp;" day(s)",IF(F20-TODAY()&lt;=14,"Due in "&amp;(F20-TODAY())&amp;" day(s)","Due "&amp;(F20-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B20="","",IF(G20&lt;=0,"Paid in full",IF(F20="","Balance due, no date set",IF(F20&lt;TODAY(),"Overdue by "&amp;TODAY()-F20&amp;IF(TODAY()-F20=1," day"," days"),IF(F20=TODAY(),"Due today",IF(F20-TODAY()&lt;=14,"Due in "&amp;F20-TODAY()&amp;IF(F20-TODAY()=1," day"," days"),"Next payment in "&amp;F20-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I20" s="1" t="n"/>
@@ -3548,7 +3564,7 @@
         <v/>
       </c>
       <c r="H21" s="33">
-        <f>IF(B21="","",IF(G21&lt;=0,"✓ Paid in full",IF(F21="","Balance, no date yet",IF(F21&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F21)&amp;" day(s)",IF(F21-TODAY()&lt;=14,"Due in "&amp;(F21-TODAY())&amp;" day(s)","Due "&amp;(F21-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B21="","",IF(G21&lt;=0,"Paid in full",IF(F21="","Balance due, no date set",IF(F21&lt;TODAY(),"Overdue by "&amp;TODAY()-F21&amp;IF(TODAY()-F21=1," day"," days"),IF(F21=TODAY(),"Due today",IF(F21-TODAY()&lt;=14,"Due in "&amp;F21-TODAY()&amp;IF(F21-TODAY()=1," day"," days"),"Next payment in "&amp;F21-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I21" s="1" t="n"/>
@@ -3565,7 +3581,7 @@
         <v/>
       </c>
       <c r="H22" s="33">
-        <f>IF(B22="","",IF(G22&lt;=0,"✓ Paid in full",IF(F22="","Balance, no date yet",IF(F22&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F22)&amp;" day(s)",IF(F22-TODAY()&lt;=14,"Due in "&amp;(F22-TODAY())&amp;" day(s)","Due "&amp;(F22-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B22="","",IF(G22&lt;=0,"Paid in full",IF(F22="","Balance due, no date set",IF(F22&lt;TODAY(),"Overdue by "&amp;TODAY()-F22&amp;IF(TODAY()-F22=1," day"," days"),IF(F22=TODAY(),"Due today",IF(F22-TODAY()&lt;=14,"Due in "&amp;F22-TODAY()&amp;IF(F22-TODAY()=1," day"," days"),"Next payment in "&amp;F22-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I22" s="1" t="n"/>
@@ -3582,7 +3598,7 @@
         <v/>
       </c>
       <c r="H23" s="33">
-        <f>IF(B23="","",IF(G23&lt;=0,"✓ Paid in full",IF(F23="","Balance, no date yet",IF(F23&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F23)&amp;" day(s)",IF(F23-TODAY()&lt;=14,"Due in "&amp;(F23-TODAY())&amp;" day(s)","Due "&amp;(F23-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B23="","",IF(G23&lt;=0,"Paid in full",IF(F23="","Balance due, no date set",IF(F23&lt;TODAY(),"Overdue by "&amp;TODAY()-F23&amp;IF(TODAY()-F23=1," day"," days"),IF(F23=TODAY(),"Due today",IF(F23-TODAY()&lt;=14,"Due in "&amp;F23-TODAY()&amp;IF(F23-TODAY()=1," day"," days"),"Next payment in "&amp;F23-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I23" s="1" t="n"/>
@@ -3599,7 +3615,7 @@
         <v/>
       </c>
       <c r="H24" s="33">
-        <f>IF(B24="","",IF(G24&lt;=0,"✓ Paid in full",IF(F24="","Balance, no date yet",IF(F24&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F24)&amp;" day(s)",IF(F24-TODAY()&lt;=14,"Due in "&amp;(F24-TODAY())&amp;" day(s)","Due "&amp;(F24-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B24="","",IF(G24&lt;=0,"Paid in full",IF(F24="","Balance due, no date set",IF(F24&lt;TODAY(),"Overdue by "&amp;TODAY()-F24&amp;IF(TODAY()-F24=1," day"," days"),IF(F24=TODAY(),"Due today",IF(F24-TODAY()&lt;=14,"Due in "&amp;F24-TODAY()&amp;IF(F24-TODAY()=1," day"," days"),"Next payment in "&amp;F24-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I24" s="1" t="n"/>
@@ -3616,7 +3632,7 @@
         <v/>
       </c>
       <c r="H25" s="33">
-        <f>IF(B25="","",IF(G25&lt;=0,"✓ Paid in full",IF(F25="","Balance, no date yet",IF(F25&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F25)&amp;" day(s)",IF(F25-TODAY()&lt;=14,"Due in "&amp;(F25-TODAY())&amp;" day(s)","Due "&amp;(F25-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B25="","",IF(G25&lt;=0,"Paid in full",IF(F25="","Balance due, no date set",IF(F25&lt;TODAY(),"Overdue by "&amp;TODAY()-F25&amp;IF(TODAY()-F25=1," day"," days"),IF(F25=TODAY(),"Due today",IF(F25-TODAY()&lt;=14,"Due in "&amp;F25-TODAY()&amp;IF(F25-TODAY()=1," day"," days"),"Next payment in "&amp;F25-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I25" s="1" t="n"/>
@@ -3633,7 +3649,7 @@
         <v/>
       </c>
       <c r="H26" s="33">
-        <f>IF(B26="","",IF(G26&lt;=0,"✓ Paid in full",IF(F26="","Balance, no date yet",IF(F26&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F26)&amp;" day(s)",IF(F26-TODAY()&lt;=14,"Due in "&amp;(F26-TODAY())&amp;" day(s)","Due "&amp;(F26-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B26="","",IF(G26&lt;=0,"Paid in full",IF(F26="","Balance due, no date set",IF(F26&lt;TODAY(),"Overdue by "&amp;TODAY()-F26&amp;IF(TODAY()-F26=1," day"," days"),IF(F26=TODAY(),"Due today",IF(F26-TODAY()&lt;=14,"Due in "&amp;F26-TODAY()&amp;IF(F26-TODAY()=1," day"," days"),"Next payment in "&amp;F26-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I26" s="1" t="n"/>
@@ -3650,7 +3666,7 @@
         <v/>
       </c>
       <c r="H27" s="33">
-        <f>IF(B27="","",IF(G27&lt;=0,"✓ Paid in full",IF(F27="","Balance, no date yet",IF(F27&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F27)&amp;" day(s)",IF(F27-TODAY()&lt;=14,"Due in "&amp;(F27-TODAY())&amp;" day(s)","Due "&amp;(F27-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B27="","",IF(G27&lt;=0,"Paid in full",IF(F27="","Balance due, no date set",IF(F27&lt;TODAY(),"Overdue by "&amp;TODAY()-F27&amp;IF(TODAY()-F27=1," day"," days"),IF(F27=TODAY(),"Due today",IF(F27-TODAY()&lt;=14,"Due in "&amp;F27-TODAY()&amp;IF(F27-TODAY()=1," day"," days"),"Next payment in "&amp;F27-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I27" s="1" t="n"/>
@@ -3667,7 +3683,7 @@
         <v/>
       </c>
       <c r="H28" s="33">
-        <f>IF(B28="","",IF(G28&lt;=0,"✓ Paid in full",IF(F28="","Balance, no date yet",IF(F28&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F28)&amp;" day(s)",IF(F28-TODAY()&lt;=14,"Due in "&amp;(F28-TODAY())&amp;" day(s)","Due "&amp;(F28-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B28="","",IF(G28&lt;=0,"Paid in full",IF(F28="","Balance due, no date set",IF(F28&lt;TODAY(),"Overdue by "&amp;TODAY()-F28&amp;IF(TODAY()-F28=1," day"," days"),IF(F28=TODAY(),"Due today",IF(F28-TODAY()&lt;=14,"Due in "&amp;F28-TODAY()&amp;IF(F28-TODAY()=1," day"," days"),"Next payment in "&amp;F28-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I28" s="1" t="n"/>
@@ -3684,7 +3700,7 @@
         <v/>
       </c>
       <c r="H29" s="33">
-        <f>IF(B29="","",IF(G29&lt;=0,"✓ Paid in full",IF(F29="","Balance, no date yet",IF(F29&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F29)&amp;" day(s)",IF(F29-TODAY()&lt;=14,"Due in "&amp;(F29-TODAY())&amp;" day(s)","Due "&amp;(F29-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B29="","",IF(G29&lt;=0,"Paid in full",IF(F29="","Balance due, no date set",IF(F29&lt;TODAY(),"Overdue by "&amp;TODAY()-F29&amp;IF(TODAY()-F29=1," day"," days"),IF(F29=TODAY(),"Due today",IF(F29-TODAY()&lt;=14,"Due in "&amp;F29-TODAY()&amp;IF(F29-TODAY()=1," day"," days"),"Next payment in "&amp;F29-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I29" s="1" t="n"/>
@@ -3701,7 +3717,7 @@
         <v/>
       </c>
       <c r="H30" s="33">
-        <f>IF(B30="","",IF(G30&lt;=0,"✓ Paid in full",IF(F30="","Balance, no date yet",IF(F30&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F30)&amp;" day(s)",IF(F30-TODAY()&lt;=14,"Due in "&amp;(F30-TODAY())&amp;" day(s)","Due "&amp;(F30-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B30="","",IF(G30&lt;=0,"Paid in full",IF(F30="","Balance due, no date set",IF(F30&lt;TODAY(),"Overdue by "&amp;TODAY()-F30&amp;IF(TODAY()-F30=1," day"," days"),IF(F30=TODAY(),"Due today",IF(F30-TODAY()&lt;=14,"Due in "&amp;F30-TODAY()&amp;IF(F30-TODAY()=1," day"," days"),"Next payment in "&amp;F30-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I30" s="1" t="n"/>
@@ -3718,7 +3734,7 @@
         <v/>
       </c>
       <c r="H31" s="33">
-        <f>IF(B31="","",IF(G31&lt;=0,"✓ Paid in full",IF(F31="","Balance, no date yet",IF(F31&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F31)&amp;" day(s)",IF(F31-TODAY()&lt;=14,"Due in "&amp;(F31-TODAY())&amp;" day(s)","Due "&amp;(F31-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B31="","",IF(G31&lt;=0,"Paid in full",IF(F31="","Balance due, no date set",IF(F31&lt;TODAY(),"Overdue by "&amp;TODAY()-F31&amp;IF(TODAY()-F31=1," day"," days"),IF(F31=TODAY(),"Due today",IF(F31-TODAY()&lt;=14,"Due in "&amp;F31-TODAY()&amp;IF(F31-TODAY()=1," day"," days"),"Next payment in "&amp;F31-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I31" s="1" t="n"/>
@@ -3735,7 +3751,7 @@
         <v/>
       </c>
       <c r="H32" s="33">
-        <f>IF(B32="","",IF(G32&lt;=0,"✓ Paid in full",IF(F32="","Balance, no date yet",IF(F32&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F32)&amp;" day(s)",IF(F32-TODAY()&lt;=14,"Due in "&amp;(F32-TODAY())&amp;" day(s)","Due "&amp;(F32-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B32="","",IF(G32&lt;=0,"Paid in full",IF(F32="","Balance due, no date set",IF(F32&lt;TODAY(),"Overdue by "&amp;TODAY()-F32&amp;IF(TODAY()-F32=1," day"," days"),IF(F32=TODAY(),"Due today",IF(F32-TODAY()&lt;=14,"Due in "&amp;F32-TODAY()&amp;IF(F32-TODAY()=1," day"," days"),"Next payment in "&amp;F32-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I32" s="1" t="n"/>
@@ -3752,7 +3768,7 @@
         <v/>
       </c>
       <c r="H33" s="33">
-        <f>IF(B33="","",IF(G33&lt;=0,"✓ Paid in full",IF(F33="","Balance, no date yet",IF(F33&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F33)&amp;" day(s)",IF(F33-TODAY()&lt;=14,"Due in "&amp;(F33-TODAY())&amp;" day(s)","Due "&amp;(F33-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B33="","",IF(G33&lt;=0,"Paid in full",IF(F33="","Balance due, no date set",IF(F33&lt;TODAY(),"Overdue by "&amp;TODAY()-F33&amp;IF(TODAY()-F33=1," day"," days"),IF(F33=TODAY(),"Due today",IF(F33-TODAY()&lt;=14,"Due in "&amp;F33-TODAY()&amp;IF(F33-TODAY()=1," day"," days"),"Next payment in "&amp;F33-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I33" s="1" t="n"/>
@@ -3769,7 +3785,7 @@
         <v/>
       </c>
       <c r="H34" s="33">
-        <f>IF(B34="","",IF(G34&lt;=0,"✓ Paid in full",IF(F34="","Balance, no date yet",IF(F34&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F34)&amp;" day(s)",IF(F34-TODAY()&lt;=14,"Due in "&amp;(F34-TODAY())&amp;" day(s)","Due "&amp;(F34-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B34="","",IF(G34&lt;=0,"Paid in full",IF(F34="","Balance due, no date set",IF(F34&lt;TODAY(),"Overdue by "&amp;TODAY()-F34&amp;IF(TODAY()-F34=1," day"," days"),IF(F34=TODAY(),"Due today",IF(F34-TODAY()&lt;=14,"Due in "&amp;F34-TODAY()&amp;IF(F34-TODAY()=1," day"," days"),"Next payment in "&amp;F34-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I34" s="1" t="n"/>
@@ -3786,7 +3802,7 @@
         <v/>
       </c>
       <c r="H35" s="33">
-        <f>IF(B35="","",IF(G35&lt;=0,"✓ Paid in full",IF(F35="","Balance, no date yet",IF(F35&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F35)&amp;" day(s)",IF(F35-TODAY()&lt;=14,"Due in "&amp;(F35-TODAY())&amp;" day(s)","Due "&amp;(F35-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B35="","",IF(G35&lt;=0,"Paid in full",IF(F35="","Balance due, no date set",IF(F35&lt;TODAY(),"Overdue by "&amp;TODAY()-F35&amp;IF(TODAY()-F35=1," day"," days"),IF(F35=TODAY(),"Due today",IF(F35-TODAY()&lt;=14,"Due in "&amp;F35-TODAY()&amp;IF(F35-TODAY()=1," day"," days"),"Next payment in "&amp;F35-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I35" s="1" t="n"/>
@@ -3803,7 +3819,7 @@
         <v/>
       </c>
       <c r="H36" s="33">
-        <f>IF(B36="","",IF(G36&lt;=0,"✓ Paid in full",IF(F36="","Balance, no date yet",IF(F36&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F36)&amp;" day(s)",IF(F36-TODAY()&lt;=14,"Due in "&amp;(F36-TODAY())&amp;" day(s)","Due "&amp;(F36-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B36="","",IF(G36&lt;=0,"Paid in full",IF(F36="","Balance due, no date set",IF(F36&lt;TODAY(),"Overdue by "&amp;TODAY()-F36&amp;IF(TODAY()-F36=1," day"," days"),IF(F36=TODAY(),"Due today",IF(F36-TODAY()&lt;=14,"Due in "&amp;F36-TODAY()&amp;IF(F36-TODAY()=1," day"," days"),"Next payment in "&amp;F36-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I36" s="1" t="n"/>
@@ -3820,7 +3836,7 @@
         <v/>
       </c>
       <c r="H37" s="33">
-        <f>IF(B37="","",IF(G37&lt;=0,"✓ Paid in full",IF(F37="","Balance, no date yet",IF(F37&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F37)&amp;" day(s)",IF(F37-TODAY()&lt;=14,"Due in "&amp;(F37-TODAY())&amp;" day(s)","Due "&amp;(F37-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B37="","",IF(G37&lt;=0,"Paid in full",IF(F37="","Balance due, no date set",IF(F37&lt;TODAY(),"Overdue by "&amp;TODAY()-F37&amp;IF(TODAY()-F37=1," day"," days"),IF(F37=TODAY(),"Due today",IF(F37-TODAY()&lt;=14,"Due in "&amp;F37-TODAY()&amp;IF(F37-TODAY()=1," day"," days"),"Next payment in "&amp;F37-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I37" s="1" t="n"/>
@@ -3837,7 +3853,7 @@
         <v/>
       </c>
       <c r="H38" s="33">
-        <f>IF(B38="","",IF(G38&lt;=0,"✓ Paid in full",IF(F38="","Balance, no date yet",IF(F38&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F38)&amp;" day(s)",IF(F38-TODAY()&lt;=14,"Due in "&amp;(F38-TODAY())&amp;" day(s)","Due "&amp;(F38-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B38="","",IF(G38&lt;=0,"Paid in full",IF(F38="","Balance due, no date set",IF(F38&lt;TODAY(),"Overdue by "&amp;TODAY()-F38&amp;IF(TODAY()-F38=1," day"," days"),IF(F38=TODAY(),"Due today",IF(F38-TODAY()&lt;=14,"Due in "&amp;F38-TODAY()&amp;IF(F38-TODAY()=1," day"," days"),"Next payment in "&amp;F38-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I38" s="1" t="n"/>
@@ -3854,7 +3870,7 @@
         <v/>
       </c>
       <c r="H39" s="33">
-        <f>IF(B39="","",IF(G39&lt;=0,"✓ Paid in full",IF(F39="","Balance, no date yet",IF(F39&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F39)&amp;" day(s)",IF(F39-TODAY()&lt;=14,"Due in "&amp;(F39-TODAY())&amp;" day(s)","Due "&amp;(F39-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B39="","",IF(G39&lt;=0,"Paid in full",IF(F39="","Balance due, no date set",IF(F39&lt;TODAY(),"Overdue by "&amp;TODAY()-F39&amp;IF(TODAY()-F39=1," day"," days"),IF(F39=TODAY(),"Due today",IF(F39-TODAY()&lt;=14,"Due in "&amp;F39-TODAY()&amp;IF(F39-TODAY()=1," day"," days"),"Next payment in "&amp;F39-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I39" s="1" t="n"/>
@@ -3871,7 +3887,7 @@
         <v/>
       </c>
       <c r="H40" s="33">
-        <f>IF(B40="","",IF(G40&lt;=0,"✓ Paid in full",IF(F40="","Balance, no date yet",IF(F40&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F40)&amp;" day(s)",IF(F40-TODAY()&lt;=14,"Due in "&amp;(F40-TODAY())&amp;" day(s)","Due "&amp;(F40-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B40="","",IF(G40&lt;=0,"Paid in full",IF(F40="","Balance due, no date set",IF(F40&lt;TODAY(),"Overdue by "&amp;TODAY()-F40&amp;IF(TODAY()-F40=1," day"," days"),IF(F40=TODAY(),"Due today",IF(F40-TODAY()&lt;=14,"Due in "&amp;F40-TODAY()&amp;IF(F40-TODAY()=1," day"," days"),"Next payment in "&amp;F40-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I40" s="1" t="n"/>
@@ -3888,7 +3904,7 @@
         <v/>
       </c>
       <c r="H41" s="33">
-        <f>IF(B41="","",IF(G41&lt;=0,"✓ Paid in full",IF(F41="","Balance, no date yet",IF(F41&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F41)&amp;" day(s)",IF(F41-TODAY()&lt;=14,"Due in "&amp;(F41-TODAY())&amp;" day(s)","Due "&amp;(F41-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B41="","",IF(G41&lt;=0,"Paid in full",IF(F41="","Balance due, no date set",IF(F41&lt;TODAY(),"Overdue by "&amp;TODAY()-F41&amp;IF(TODAY()-F41=1," day"," days"),IF(F41=TODAY(),"Due today",IF(F41-TODAY()&lt;=14,"Due in "&amp;F41-TODAY()&amp;IF(F41-TODAY()=1," day"," days"),"Next payment in "&amp;F41-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I41" s="1" t="n"/>
@@ -3905,7 +3921,7 @@
         <v/>
       </c>
       <c r="H42" s="33">
-        <f>IF(B42="","",IF(G42&lt;=0,"✓ Paid in full",IF(F42="","Balance, no date yet",IF(F42&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F42)&amp;" day(s)",IF(F42-TODAY()&lt;=14,"Due in "&amp;(F42-TODAY())&amp;" day(s)","Due "&amp;(F42-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B42="","",IF(G42&lt;=0,"Paid in full",IF(F42="","Balance due, no date set",IF(F42&lt;TODAY(),"Overdue by "&amp;TODAY()-F42&amp;IF(TODAY()-F42=1," day"," days"),IF(F42=TODAY(),"Due today",IF(F42-TODAY()&lt;=14,"Due in "&amp;F42-TODAY()&amp;IF(F42-TODAY()=1," day"," days"),"Next payment in "&amp;F42-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I42" s="1" t="n"/>
@@ -3922,7 +3938,7 @@
         <v/>
       </c>
       <c r="H43" s="33">
-        <f>IF(B43="","",IF(G43&lt;=0,"✓ Paid in full",IF(F43="","Balance, no date yet",IF(F43&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F43)&amp;" day(s)",IF(F43-TODAY()&lt;=14,"Due in "&amp;(F43-TODAY())&amp;" day(s)","Due "&amp;(F43-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B43="","",IF(G43&lt;=0,"Paid in full",IF(F43="","Balance due, no date set",IF(F43&lt;TODAY(),"Overdue by "&amp;TODAY()-F43&amp;IF(TODAY()-F43=1," day"," days"),IF(F43=TODAY(),"Due today",IF(F43-TODAY()&lt;=14,"Due in "&amp;F43-TODAY()&amp;IF(F43-TODAY()=1," day"," days"),"Next payment in "&amp;F43-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I43" s="1" t="n"/>
@@ -3939,7 +3955,7 @@
         <v/>
       </c>
       <c r="H44" s="33">
-        <f>IF(B44="","",IF(G44&lt;=0,"✓ Paid in full",IF(F44="","Balance, no date yet",IF(F44&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F44)&amp;" day(s)",IF(F44-TODAY()&lt;=14,"Due in "&amp;(F44-TODAY())&amp;" day(s)","Due "&amp;(F44-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B44="","",IF(G44&lt;=0,"Paid in full",IF(F44="","Balance due, no date set",IF(F44&lt;TODAY(),"Overdue by "&amp;TODAY()-F44&amp;IF(TODAY()-F44=1," day"," days"),IF(F44=TODAY(),"Due today",IF(F44-TODAY()&lt;=14,"Due in "&amp;F44-TODAY()&amp;IF(F44-TODAY()=1," day"," days"),"Next payment in "&amp;F44-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I44" s="1" t="n"/>
@@ -3956,7 +3972,7 @@
         <v/>
       </c>
       <c r="H45" s="33">
-        <f>IF(B45="","",IF(G45&lt;=0,"✓ Paid in full",IF(F45="","Balance, no date yet",IF(F45&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F45)&amp;" day(s)",IF(F45-TODAY()&lt;=14,"Due in "&amp;(F45-TODAY())&amp;" day(s)","Due "&amp;(F45-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B45="","",IF(G45&lt;=0,"Paid in full",IF(F45="","Balance due, no date set",IF(F45&lt;TODAY(),"Overdue by "&amp;TODAY()-F45&amp;IF(TODAY()-F45=1," day"," days"),IF(F45=TODAY(),"Due today",IF(F45-TODAY()&lt;=14,"Due in "&amp;F45-TODAY()&amp;IF(F45-TODAY()=1," day"," days"),"Next payment in "&amp;F45-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I45" s="1" t="n"/>
@@ -3973,7 +3989,7 @@
         <v/>
       </c>
       <c r="H46" s="33">
-        <f>IF(B46="","",IF(G46&lt;=0,"✓ Paid in full",IF(F46="","Balance, no date yet",IF(F46&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F46)&amp;" day(s)",IF(F46-TODAY()&lt;=14,"Due in "&amp;(F46-TODAY())&amp;" day(s)","Due "&amp;(F46-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B46="","",IF(G46&lt;=0,"Paid in full",IF(F46="","Balance due, no date set",IF(F46&lt;TODAY(),"Overdue by "&amp;TODAY()-F46&amp;IF(TODAY()-F46=1," day"," days"),IF(F46=TODAY(),"Due today",IF(F46-TODAY()&lt;=14,"Due in "&amp;F46-TODAY()&amp;IF(F46-TODAY()=1," day"," days"),"Next payment in "&amp;F46-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I46" s="1" t="n"/>
@@ -3990,7 +4006,7 @@
         <v/>
       </c>
       <c r="H47" s="33">
-        <f>IF(B47="","",IF(G47&lt;=0,"✓ Paid in full",IF(F47="","Balance, no date yet",IF(F47&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F47)&amp;" day(s)",IF(F47-TODAY()&lt;=14,"Due in "&amp;(F47-TODAY())&amp;" day(s)","Due "&amp;(F47-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B47="","",IF(G47&lt;=0,"Paid in full",IF(F47="","Balance due, no date set",IF(F47&lt;TODAY(),"Overdue by "&amp;TODAY()-F47&amp;IF(TODAY()-F47=1," day"," days"),IF(F47=TODAY(),"Due today",IF(F47-TODAY()&lt;=14,"Due in "&amp;F47-TODAY()&amp;IF(F47-TODAY()=1," day"," days"),"Next payment in "&amp;F47-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I47" s="1" t="n"/>
@@ -4007,7 +4023,7 @@
         <v/>
       </c>
       <c r="H48" s="33">
-        <f>IF(B48="","",IF(G48&lt;=0,"✓ Paid in full",IF(F48="","Balance, no date yet",IF(F48&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F48)&amp;" day(s)",IF(F48-TODAY()&lt;=14,"Due in "&amp;(F48-TODAY())&amp;" day(s)","Due "&amp;(F48-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B48="","",IF(G48&lt;=0,"Paid in full",IF(F48="","Balance due, no date set",IF(F48&lt;TODAY(),"Overdue by "&amp;TODAY()-F48&amp;IF(TODAY()-F48=1," day"," days"),IF(F48=TODAY(),"Due today",IF(F48-TODAY()&lt;=14,"Due in "&amp;F48-TODAY()&amp;IF(F48-TODAY()=1," day"," days"),"Next payment in "&amp;F48-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I48" s="1" t="n"/>
@@ -4024,7 +4040,7 @@
         <v/>
       </c>
       <c r="H49" s="33">
-        <f>IF(B49="","",IF(G49&lt;=0,"✓ Paid in full",IF(F49="","Balance, no date yet",IF(F49&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F49)&amp;" day(s)",IF(F49-TODAY()&lt;=14,"Due in "&amp;(F49-TODAY())&amp;" day(s)","Due "&amp;(F49-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B49="","",IF(G49&lt;=0,"Paid in full",IF(F49="","Balance due, no date set",IF(F49&lt;TODAY(),"Overdue by "&amp;TODAY()-F49&amp;IF(TODAY()-F49=1," day"," days"),IF(F49=TODAY(),"Due today",IF(F49-TODAY()&lt;=14,"Due in "&amp;F49-TODAY()&amp;IF(F49-TODAY()=1," day"," days"),"Next payment in "&amp;F49-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I49" s="1" t="n"/>
@@ -4041,7 +4057,7 @@
         <v/>
       </c>
       <c r="H50" s="33">
-        <f>IF(B50="","",IF(G50&lt;=0,"✓ Paid in full",IF(F50="","Balance, no date yet",IF(F50&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F50)&amp;" day(s)",IF(F50-TODAY()&lt;=14,"Due in "&amp;(F50-TODAY())&amp;" day(s)","Due "&amp;(F50-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B50="","",IF(G50&lt;=0,"Paid in full",IF(F50="","Balance due, no date set",IF(F50&lt;TODAY(),"Overdue by "&amp;TODAY()-F50&amp;IF(TODAY()-F50=1," day"," days"),IF(F50=TODAY(),"Due today",IF(F50-TODAY()&lt;=14,"Due in "&amp;F50-TODAY()&amp;IF(F50-TODAY()=1," day"," days"),"Next payment in "&amp;F50-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I50" s="1" t="n"/>
@@ -4058,7 +4074,7 @@
         <v/>
       </c>
       <c r="H51" s="33">
-        <f>IF(B51="","",IF(G51&lt;=0,"✓ Paid in full",IF(F51="","Balance, no date yet",IF(F51&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F51)&amp;" day(s)",IF(F51-TODAY()&lt;=14,"Due in "&amp;(F51-TODAY())&amp;" day(s)","Due "&amp;(F51-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B51="","",IF(G51&lt;=0,"Paid in full",IF(F51="","Balance due, no date set",IF(F51&lt;TODAY(),"Overdue by "&amp;TODAY()-F51&amp;IF(TODAY()-F51=1," day"," days"),IF(F51=TODAY(),"Due today",IF(F51-TODAY()&lt;=14,"Due in "&amp;F51-TODAY()&amp;IF(F51-TODAY()=1," day"," days"),"Next payment in "&amp;F51-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I51" s="1" t="n"/>
@@ -4075,7 +4091,7 @@
         <v/>
       </c>
       <c r="H52" s="33">
-        <f>IF(B52="","",IF(G52&lt;=0,"✓ Paid in full",IF(F52="","Balance, no date yet",IF(F52&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F52)&amp;" day(s)",IF(F52-TODAY()&lt;=14,"Due in "&amp;(F52-TODAY())&amp;" day(s)","Due "&amp;(F52-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B52="","",IF(G52&lt;=0,"Paid in full",IF(F52="","Balance due, no date set",IF(F52&lt;TODAY(),"Overdue by "&amp;TODAY()-F52&amp;IF(TODAY()-F52=1," day"," days"),IF(F52=TODAY(),"Due today",IF(F52-TODAY()&lt;=14,"Due in "&amp;F52-TODAY()&amp;IF(F52-TODAY()=1," day"," days"),"Next payment in "&amp;F52-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I52" s="1" t="n"/>
@@ -4092,7 +4108,7 @@
         <v/>
       </c>
       <c r="H53" s="33">
-        <f>IF(B53="","",IF(G53&lt;=0,"✓ Paid in full",IF(F53="","Balance, no date yet",IF(F53&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F53)&amp;" day(s)",IF(F53-TODAY()&lt;=14,"Due in "&amp;(F53-TODAY())&amp;" day(s)","Due "&amp;(F53-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B53="","",IF(G53&lt;=0,"Paid in full",IF(F53="","Balance due, no date set",IF(F53&lt;TODAY(),"Overdue by "&amp;TODAY()-F53&amp;IF(TODAY()-F53=1," day"," days"),IF(F53=TODAY(),"Due today",IF(F53-TODAY()&lt;=14,"Due in "&amp;F53-TODAY()&amp;IF(F53-TODAY()=1," day"," days"),"Next payment in "&amp;F53-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I53" s="1" t="n"/>
@@ -4109,7 +4125,7 @@
         <v/>
       </c>
       <c r="H54" s="33">
-        <f>IF(B54="","",IF(G54&lt;=0,"✓ Paid in full",IF(F54="","Balance, no date yet",IF(F54&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F54)&amp;" day(s)",IF(F54-TODAY()&lt;=14,"Due in "&amp;(F54-TODAY())&amp;" day(s)","Due "&amp;(F54-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B54="","",IF(G54&lt;=0,"Paid in full",IF(F54="","Balance due, no date set",IF(F54&lt;TODAY(),"Overdue by "&amp;TODAY()-F54&amp;IF(TODAY()-F54=1," day"," days"),IF(F54=TODAY(),"Due today",IF(F54-TODAY()&lt;=14,"Due in "&amp;F54-TODAY()&amp;IF(F54-TODAY()=1," day"," days"),"Next payment in "&amp;F54-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I54" s="1" t="n"/>
@@ -4126,7 +4142,7 @@
         <v/>
       </c>
       <c r="H55" s="33">
-        <f>IF(B55="","",IF(G55&lt;=0,"✓ Paid in full",IF(F55="","Balance, no date yet",IF(F55&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F55)&amp;" day(s)",IF(F55-TODAY()&lt;=14,"Due in "&amp;(F55-TODAY())&amp;" day(s)","Due "&amp;(F55-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B55="","",IF(G55&lt;=0,"Paid in full",IF(F55="","Balance due, no date set",IF(F55&lt;TODAY(),"Overdue by "&amp;TODAY()-F55&amp;IF(TODAY()-F55=1," day"," days"),IF(F55=TODAY(),"Due today",IF(F55-TODAY()&lt;=14,"Due in "&amp;F55-TODAY()&amp;IF(F55-TODAY()=1," day"," days"),"Next payment in "&amp;F55-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I55" s="1" t="n"/>
@@ -4143,7 +4159,7 @@
         <v/>
       </c>
       <c r="H56" s="33">
-        <f>IF(B56="","",IF(G56&lt;=0,"✓ Paid in full",IF(F56="","Balance, no date yet",IF(F56&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F56)&amp;" day(s)",IF(F56-TODAY()&lt;=14,"Due in "&amp;(F56-TODAY())&amp;" day(s)","Due "&amp;(F56-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B56="","",IF(G56&lt;=0,"Paid in full",IF(F56="","Balance due, no date set",IF(F56&lt;TODAY(),"Overdue by "&amp;TODAY()-F56&amp;IF(TODAY()-F56=1," day"," days"),IF(F56=TODAY(),"Due today",IF(F56-TODAY()&lt;=14,"Due in "&amp;F56-TODAY()&amp;IF(F56-TODAY()=1," day"," days"),"Next payment in "&amp;F56-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I56" s="1" t="n"/>
@@ -4160,7 +4176,7 @@
         <v/>
       </c>
       <c r="H57" s="33">
-        <f>IF(B57="","",IF(G57&lt;=0,"✓ Paid in full",IF(F57="","Balance, no date yet",IF(F57&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F57)&amp;" day(s)",IF(F57-TODAY()&lt;=14,"Due in "&amp;(F57-TODAY())&amp;" day(s)","Due "&amp;(F57-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B57="","",IF(G57&lt;=0,"Paid in full",IF(F57="","Balance due, no date set",IF(F57&lt;TODAY(),"Overdue by "&amp;TODAY()-F57&amp;IF(TODAY()-F57=1," day"," days"),IF(F57=TODAY(),"Due today",IF(F57-TODAY()&lt;=14,"Due in "&amp;F57-TODAY()&amp;IF(F57-TODAY()=1," day"," days"),"Next payment in "&amp;F57-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I57" s="1" t="n"/>
@@ -4177,7 +4193,7 @@
         <v/>
       </c>
       <c r="H58" s="33">
-        <f>IF(B58="","",IF(G58&lt;=0,"✓ Paid in full",IF(F58="","Balance, no date yet",IF(F58&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F58)&amp;" day(s)",IF(F58-TODAY()&lt;=14,"Due in "&amp;(F58-TODAY())&amp;" day(s)","Due "&amp;(F58-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B58="","",IF(G58&lt;=0,"Paid in full",IF(F58="","Balance due, no date set",IF(F58&lt;TODAY(),"Overdue by "&amp;TODAY()-F58&amp;IF(TODAY()-F58=1," day"," days"),IF(F58=TODAY(),"Due today",IF(F58-TODAY()&lt;=14,"Due in "&amp;F58-TODAY()&amp;IF(F58-TODAY()=1," day"," days"),"Next payment in "&amp;F58-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I58" s="1" t="n"/>
@@ -4194,7 +4210,7 @@
         <v/>
       </c>
       <c r="H59" s="33">
-        <f>IF(B59="","",IF(G59&lt;=0,"✓ Paid in full",IF(F59="","Balance, no date yet",IF(F59&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F59)&amp;" day(s)",IF(F59-TODAY()&lt;=14,"Due in "&amp;(F59-TODAY())&amp;" day(s)","Due "&amp;(F59-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B59="","",IF(G59&lt;=0,"Paid in full",IF(F59="","Balance due, no date set",IF(F59&lt;TODAY(),"Overdue by "&amp;TODAY()-F59&amp;IF(TODAY()-F59=1," day"," days"),IF(F59=TODAY(),"Due today",IF(F59-TODAY()&lt;=14,"Due in "&amp;F59-TODAY()&amp;IF(F59-TODAY()=1," day"," days"),"Next payment in "&amp;F59-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I59" s="1" t="n"/>
@@ -4211,7 +4227,7 @@
         <v/>
       </c>
       <c r="H60" s="33">
-        <f>IF(B60="","",IF(G60&lt;=0,"✓ Paid in full",IF(F60="","Balance, no date yet",IF(F60&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F60)&amp;" day(s)",IF(F60-TODAY()&lt;=14,"Due in "&amp;(F60-TODAY())&amp;" day(s)","Due "&amp;(F60-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B60="","",IF(G60&lt;=0,"Paid in full",IF(F60="","Balance due, no date set",IF(F60&lt;TODAY(),"Overdue by "&amp;TODAY()-F60&amp;IF(TODAY()-F60=1," day"," days"),IF(F60=TODAY(),"Due today",IF(F60-TODAY()&lt;=14,"Due in "&amp;F60-TODAY()&amp;IF(F60-TODAY()=1," day"," days"),"Next payment in "&amp;F60-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I60" s="1" t="n"/>
@@ -4228,7 +4244,7 @@
         <v/>
       </c>
       <c r="H61" s="33">
-        <f>IF(B61="","",IF(G61&lt;=0,"✓ Paid in full",IF(F61="","Balance, no date yet",IF(F61&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F61)&amp;" day(s)",IF(F61-TODAY()&lt;=14,"Due in "&amp;(F61-TODAY())&amp;" day(s)","Due "&amp;(F61-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B61="","",IF(G61&lt;=0,"Paid in full",IF(F61="","Balance due, no date set",IF(F61&lt;TODAY(),"Overdue by "&amp;TODAY()-F61&amp;IF(TODAY()-F61=1," day"," days"),IF(F61=TODAY(),"Due today",IF(F61-TODAY()&lt;=14,"Due in "&amp;F61-TODAY()&amp;IF(F61-TODAY()=1," day"," days"),"Next payment in "&amp;F61-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I61" s="1" t="n"/>
@@ -4245,7 +4261,7 @@
         <v/>
       </c>
       <c r="H62" s="33">
-        <f>IF(B62="","",IF(G62&lt;=0,"✓ Paid in full",IF(F62="","Balance, no date yet",IF(F62&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F62)&amp;" day(s)",IF(F62-TODAY()&lt;=14,"Due in "&amp;(F62-TODAY())&amp;" day(s)","Due "&amp;(F62-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B62="","",IF(G62&lt;=0,"Paid in full",IF(F62="","Balance due, no date set",IF(F62&lt;TODAY(),"Overdue by "&amp;TODAY()-F62&amp;IF(TODAY()-F62=1," day"," days"),IF(F62=TODAY(),"Due today",IF(F62-TODAY()&lt;=14,"Due in "&amp;F62-TODAY()&amp;IF(F62-TODAY()=1," day"," days"),"Next payment in "&amp;F62-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I62" s="1" t="n"/>
@@ -4262,7 +4278,7 @@
         <v/>
       </c>
       <c r="H63" s="33">
-        <f>IF(B63="","",IF(G63&lt;=0,"✓ Paid in full",IF(F63="","Balance, no date yet",IF(F63&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F63)&amp;" day(s)",IF(F63-TODAY()&lt;=14,"Due in "&amp;(F63-TODAY())&amp;" day(s)","Due "&amp;(F63-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B63="","",IF(G63&lt;=0,"Paid in full",IF(F63="","Balance due, no date set",IF(F63&lt;TODAY(),"Overdue by "&amp;TODAY()-F63&amp;IF(TODAY()-F63=1," day"," days"),IF(F63=TODAY(),"Due today",IF(F63-TODAY()&lt;=14,"Due in "&amp;F63-TODAY()&amp;IF(F63-TODAY()=1," day"," days"),"Next payment in "&amp;F63-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I63" s="1" t="n"/>
@@ -4279,7 +4295,7 @@
         <v/>
       </c>
       <c r="H64" s="33">
-        <f>IF(B64="","",IF(G64&lt;=0,"✓ Paid in full",IF(F64="","Balance, no date yet",IF(F64&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F64)&amp;" day(s)",IF(F64-TODAY()&lt;=14,"Due in "&amp;(F64-TODAY())&amp;" day(s)","Due "&amp;(F64-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B64="","",IF(G64&lt;=0,"Paid in full",IF(F64="","Balance due, no date set",IF(F64&lt;TODAY(),"Overdue by "&amp;TODAY()-F64&amp;IF(TODAY()-F64=1," day"," days"),IF(F64=TODAY(),"Due today",IF(F64-TODAY()&lt;=14,"Due in "&amp;F64-TODAY()&amp;IF(F64-TODAY()=1," day"," days"),"Next payment in "&amp;F64-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I64" s="1" t="n"/>
@@ -4296,7 +4312,7 @@
         <v/>
       </c>
       <c r="H65" s="33">
-        <f>IF(B65="","",IF(G65&lt;=0,"✓ Paid in full",IF(F65="","Balance, no date yet",IF(F65&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F65)&amp;" day(s)",IF(F65-TODAY()&lt;=14,"Due in "&amp;(F65-TODAY())&amp;" day(s)","Due "&amp;(F65-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B65="","",IF(G65&lt;=0,"Paid in full",IF(F65="","Balance due, no date set",IF(F65&lt;TODAY(),"Overdue by "&amp;TODAY()-F65&amp;IF(TODAY()-F65=1," day"," days"),IF(F65=TODAY(),"Due today",IF(F65-TODAY()&lt;=14,"Due in "&amp;F65-TODAY()&amp;IF(F65-TODAY()=1," day"," days"),"Next payment in "&amp;F65-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I65" s="1" t="n"/>
@@ -4313,7 +4329,7 @@
         <v/>
       </c>
       <c r="H66" s="33">
-        <f>IF(B66="","",IF(G66&lt;=0,"✓ Paid in full",IF(F66="","Balance, no date yet",IF(F66&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F66)&amp;" day(s)",IF(F66-TODAY()&lt;=14,"Due in "&amp;(F66-TODAY())&amp;" day(s)","Due "&amp;(F66-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B66="","",IF(G66&lt;=0,"Paid in full",IF(F66="","Balance due, no date set",IF(F66&lt;TODAY(),"Overdue by "&amp;TODAY()-F66&amp;IF(TODAY()-F66=1," day"," days"),IF(F66=TODAY(),"Due today",IF(F66-TODAY()&lt;=14,"Due in "&amp;F66-TODAY()&amp;IF(F66-TODAY()=1," day"," days"),"Next payment in "&amp;F66-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I66" s="1" t="n"/>
@@ -4330,7 +4346,7 @@
         <v/>
       </c>
       <c r="H67" s="33">
-        <f>IF(B67="","",IF(G67&lt;=0,"✓ Paid in full",IF(F67="","Balance, no date yet",IF(F67&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F67)&amp;" day(s)",IF(F67-TODAY()&lt;=14,"Due in "&amp;(F67-TODAY())&amp;" day(s)","Due "&amp;(F67-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B67="","",IF(G67&lt;=0,"Paid in full",IF(F67="","Balance due, no date set",IF(F67&lt;TODAY(),"Overdue by "&amp;TODAY()-F67&amp;IF(TODAY()-F67=1," day"," days"),IF(F67=TODAY(),"Due today",IF(F67-TODAY()&lt;=14,"Due in "&amp;F67-TODAY()&amp;IF(F67-TODAY()=1," day"," days"),"Next payment in "&amp;F67-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I67" s="1" t="n"/>
@@ -4347,7 +4363,7 @@
         <v/>
       </c>
       <c r="H68" s="33">
-        <f>IF(B68="","",IF(G68&lt;=0,"✓ Paid in full",IF(F68="","Balance, no date yet",IF(F68&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F68)&amp;" day(s)",IF(F68-TODAY()&lt;=14,"Due in "&amp;(F68-TODAY())&amp;" day(s)","Due "&amp;(F68-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B68="","",IF(G68&lt;=0,"Paid in full",IF(F68="","Balance due, no date set",IF(F68&lt;TODAY(),"Overdue by "&amp;TODAY()-F68&amp;IF(TODAY()-F68=1," day"," days"),IF(F68=TODAY(),"Due today",IF(F68-TODAY()&lt;=14,"Due in "&amp;F68-TODAY()&amp;IF(F68-TODAY()=1," day"," days"),"Next payment in "&amp;F68-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I68" s="1" t="n"/>
@@ -4364,7 +4380,7 @@
         <v/>
       </c>
       <c r="H69" s="33">
-        <f>IF(B69="","",IF(G69&lt;=0,"✓ Paid in full",IF(F69="","Balance, no date yet",IF(F69&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F69)&amp;" day(s)",IF(F69-TODAY()&lt;=14,"Due in "&amp;(F69-TODAY())&amp;" day(s)","Due "&amp;(F69-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B69="","",IF(G69&lt;=0,"Paid in full",IF(F69="","Balance due, no date set",IF(F69&lt;TODAY(),"Overdue by "&amp;TODAY()-F69&amp;IF(TODAY()-F69=1," day"," days"),IF(F69=TODAY(),"Due today",IF(F69-TODAY()&lt;=14,"Due in "&amp;F69-TODAY()&amp;IF(F69-TODAY()=1," day"," days"),"Next payment in "&amp;F69-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I69" s="1" t="n"/>
@@ -4381,7 +4397,7 @@
         <v/>
       </c>
       <c r="H70" s="33">
-        <f>IF(B70="","",IF(G70&lt;=0,"✓ Paid in full",IF(F70="","Balance, no date yet",IF(F70&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F70)&amp;" day(s)",IF(F70-TODAY()&lt;=14,"Due in "&amp;(F70-TODAY())&amp;" day(s)","Due "&amp;(F70-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B70="","",IF(G70&lt;=0,"Paid in full",IF(F70="","Balance due, no date set",IF(F70&lt;TODAY(),"Overdue by "&amp;TODAY()-F70&amp;IF(TODAY()-F70=1," day"," days"),IF(F70=TODAY(),"Due today",IF(F70-TODAY()&lt;=14,"Due in "&amp;F70-TODAY()&amp;IF(F70-TODAY()=1," day"," days"),"Next payment in "&amp;F70-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I70" s="1" t="n"/>
@@ -4398,7 +4414,7 @@
         <v/>
       </c>
       <c r="H71" s="33">
-        <f>IF(B71="","",IF(G71&lt;=0,"✓ Paid in full",IF(F71="","Balance, no date yet",IF(F71&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F71)&amp;" day(s)",IF(F71-TODAY()&lt;=14,"Due in "&amp;(F71-TODAY())&amp;" day(s)","Due "&amp;(F71-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B71="","",IF(G71&lt;=0,"Paid in full",IF(F71="","Balance due, no date set",IF(F71&lt;TODAY(),"Overdue by "&amp;TODAY()-F71&amp;IF(TODAY()-F71=1," day"," days"),IF(F71=TODAY(),"Due today",IF(F71-TODAY()&lt;=14,"Due in "&amp;F71-TODAY()&amp;IF(F71-TODAY()=1," day"," days"),"Next payment in "&amp;F71-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I71" s="1" t="n"/>
@@ -4415,7 +4431,7 @@
         <v/>
       </c>
       <c r="H72" s="33">
-        <f>IF(B72="","",IF(G72&lt;=0,"✓ Paid in full",IF(F72="","Balance, no date yet",IF(F72&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F72)&amp;" day(s)",IF(F72-TODAY()&lt;=14,"Due in "&amp;(F72-TODAY())&amp;" day(s)","Due "&amp;(F72-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B72="","",IF(G72&lt;=0,"Paid in full",IF(F72="","Balance due, no date set",IF(F72&lt;TODAY(),"Overdue by "&amp;TODAY()-F72&amp;IF(TODAY()-F72=1," day"," days"),IF(F72=TODAY(),"Due today",IF(F72-TODAY()&lt;=14,"Due in "&amp;F72-TODAY()&amp;IF(F72-TODAY()=1," day"," days"),"Next payment in "&amp;F72-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I72" s="1" t="n"/>
@@ -4432,7 +4448,7 @@
         <v/>
       </c>
       <c r="H73" s="33">
-        <f>IF(B73="","",IF(G73&lt;=0,"✓ Paid in full",IF(F73="","Balance, no date yet",IF(F73&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F73)&amp;" day(s)",IF(F73-TODAY()&lt;=14,"Due in "&amp;(F73-TODAY())&amp;" day(s)","Due "&amp;(F73-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B73="","",IF(G73&lt;=0,"Paid in full",IF(F73="","Balance due, no date set",IF(F73&lt;TODAY(),"Overdue by "&amp;TODAY()-F73&amp;IF(TODAY()-F73=1," day"," days"),IF(F73=TODAY(),"Due today",IF(F73-TODAY()&lt;=14,"Due in "&amp;F73-TODAY()&amp;IF(F73-TODAY()=1," day"," days"),"Next payment in "&amp;F73-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I73" s="1" t="n"/>
@@ -4449,7 +4465,7 @@
         <v/>
       </c>
       <c r="H74" s="33">
-        <f>IF(B74="","",IF(G74&lt;=0,"✓ Paid in full",IF(F74="","Balance, no date yet",IF(F74&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F74)&amp;" day(s)",IF(F74-TODAY()&lt;=14,"Due in "&amp;(F74-TODAY())&amp;" day(s)","Due "&amp;(F74-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B74="","",IF(G74&lt;=0,"Paid in full",IF(F74="","Balance due, no date set",IF(F74&lt;TODAY(),"Overdue by "&amp;TODAY()-F74&amp;IF(TODAY()-F74=1," day"," days"),IF(F74=TODAY(),"Due today",IF(F74-TODAY()&lt;=14,"Due in "&amp;F74-TODAY()&amp;IF(F74-TODAY()=1," day"," days"),"Next payment in "&amp;F74-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I74" s="1" t="n"/>
@@ -4466,7 +4482,7 @@
         <v/>
       </c>
       <c r="H75" s="33">
-        <f>IF(B75="","",IF(G75&lt;=0,"✓ Paid in full",IF(F75="","Balance, no date yet",IF(F75&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F75)&amp;" day(s)",IF(F75-TODAY()&lt;=14,"Due in "&amp;(F75-TODAY())&amp;" day(s)","Due "&amp;(F75-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B75="","",IF(G75&lt;=0,"Paid in full",IF(F75="","Balance due, no date set",IF(F75&lt;TODAY(),"Overdue by "&amp;TODAY()-F75&amp;IF(TODAY()-F75=1," day"," days"),IF(F75=TODAY(),"Due today",IF(F75-TODAY()&lt;=14,"Due in "&amp;F75-TODAY()&amp;IF(F75-TODAY()=1," day"," days"),"Next payment in "&amp;F75-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I75" s="1" t="n"/>
@@ -4483,7 +4499,7 @@
         <v/>
       </c>
       <c r="H76" s="33">
-        <f>IF(B76="","",IF(G76&lt;=0,"✓ Paid in full",IF(F76="","Balance, no date yet",IF(F76&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F76)&amp;" day(s)",IF(F76-TODAY()&lt;=14,"Due in "&amp;(F76-TODAY())&amp;" day(s)","Due "&amp;(F76-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B76="","",IF(G76&lt;=0,"Paid in full",IF(F76="","Balance due, no date set",IF(F76&lt;TODAY(),"Overdue by "&amp;TODAY()-F76&amp;IF(TODAY()-F76=1," day"," days"),IF(F76=TODAY(),"Due today",IF(F76-TODAY()&lt;=14,"Due in "&amp;F76-TODAY()&amp;IF(F76-TODAY()=1," day"," days"),"Next payment in "&amp;F76-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I76" s="1" t="n"/>
@@ -4500,7 +4516,7 @@
         <v/>
       </c>
       <c r="H77" s="33">
-        <f>IF(B77="","",IF(G77&lt;=0,"✓ Paid in full",IF(F77="","Balance, no date yet",IF(F77&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F77)&amp;" day(s)",IF(F77-TODAY()&lt;=14,"Due in "&amp;(F77-TODAY())&amp;" day(s)","Due "&amp;(F77-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B77="","",IF(G77&lt;=0,"Paid in full",IF(F77="","Balance due, no date set",IF(F77&lt;TODAY(),"Overdue by "&amp;TODAY()-F77&amp;IF(TODAY()-F77=1," day"," days"),IF(F77=TODAY(),"Due today",IF(F77-TODAY()&lt;=14,"Due in "&amp;F77-TODAY()&amp;IF(F77-TODAY()=1," day"," days"),"Next payment in "&amp;F77-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I77" s="1" t="n"/>
@@ -4517,7 +4533,7 @@
         <v/>
       </c>
       <c r="H78" s="33">
-        <f>IF(B78="","",IF(G78&lt;=0,"✓ Paid in full",IF(F78="","Balance, no date yet",IF(F78&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F78)&amp;" day(s)",IF(F78-TODAY()&lt;=14,"Due in "&amp;(F78-TODAY())&amp;" day(s)","Due "&amp;(F78-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B78="","",IF(G78&lt;=0,"Paid in full",IF(F78="","Balance due, no date set",IF(F78&lt;TODAY(),"Overdue by "&amp;TODAY()-F78&amp;IF(TODAY()-F78=1," day"," days"),IF(F78=TODAY(),"Due today",IF(F78-TODAY()&lt;=14,"Due in "&amp;F78-TODAY()&amp;IF(F78-TODAY()=1," day"," days"),"Next payment in "&amp;F78-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I78" s="1" t="n"/>
@@ -4534,7 +4550,7 @@
         <v/>
       </c>
       <c r="H79" s="33">
-        <f>IF(B79="","",IF(G79&lt;=0,"✓ Paid in full",IF(F79="","Balance, no date yet",IF(F79&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F79)&amp;" day(s)",IF(F79-TODAY()&lt;=14,"Due in "&amp;(F79-TODAY())&amp;" day(s)","Due "&amp;(F79-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B79="","",IF(G79&lt;=0,"Paid in full",IF(F79="","Balance due, no date set",IF(F79&lt;TODAY(),"Overdue by "&amp;TODAY()-F79&amp;IF(TODAY()-F79=1," day"," days"),IF(F79=TODAY(),"Due today",IF(F79-TODAY()&lt;=14,"Due in "&amp;F79-TODAY()&amp;IF(F79-TODAY()=1," day"," days"),"Next payment in "&amp;F79-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I79" s="1" t="n"/>
@@ -4551,7 +4567,7 @@
         <v/>
       </c>
       <c r="H80" s="33">
-        <f>IF(B80="","",IF(G80&lt;=0,"✓ Paid in full",IF(F80="","Balance, no date yet",IF(F80&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F80)&amp;" day(s)",IF(F80-TODAY()&lt;=14,"Due in "&amp;(F80-TODAY())&amp;" day(s)","Due "&amp;(F80-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B80="","",IF(G80&lt;=0,"Paid in full",IF(F80="","Balance due, no date set",IF(F80&lt;TODAY(),"Overdue by "&amp;TODAY()-F80&amp;IF(TODAY()-F80=1," day"," days"),IF(F80=TODAY(),"Due today",IF(F80-TODAY()&lt;=14,"Due in "&amp;F80-TODAY()&amp;IF(F80-TODAY()=1," day"," days"),"Next payment in "&amp;F80-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I80" s="1" t="n"/>
@@ -4568,7 +4584,7 @@
         <v/>
       </c>
       <c r="H81" s="33">
-        <f>IF(B81="","",IF(G81&lt;=0,"✓ Paid in full",IF(F81="","Balance, no date yet",IF(F81&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F81)&amp;" day(s)",IF(F81-TODAY()&lt;=14,"Due in "&amp;(F81-TODAY())&amp;" day(s)","Due "&amp;(F81-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B81="","",IF(G81&lt;=0,"Paid in full",IF(F81="","Balance due, no date set",IF(F81&lt;TODAY(),"Overdue by "&amp;TODAY()-F81&amp;IF(TODAY()-F81=1," day"," days"),IF(F81=TODAY(),"Due today",IF(F81-TODAY()&lt;=14,"Due in "&amp;F81-TODAY()&amp;IF(F81-TODAY()=1," day"," days"),"Next payment in "&amp;F81-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I81" s="1" t="n"/>
@@ -4585,7 +4601,7 @@
         <v/>
       </c>
       <c r="H82" s="33">
-        <f>IF(B82="","",IF(G82&lt;=0,"✓ Paid in full",IF(F82="","Balance, no date yet",IF(F82&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F82)&amp;" day(s)",IF(F82-TODAY()&lt;=14,"Due in "&amp;(F82-TODAY())&amp;" day(s)","Due "&amp;(F82-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B82="","",IF(G82&lt;=0,"Paid in full",IF(F82="","Balance due, no date set",IF(F82&lt;TODAY(),"Overdue by "&amp;TODAY()-F82&amp;IF(TODAY()-F82=1," day"," days"),IF(F82=TODAY(),"Due today",IF(F82-TODAY()&lt;=14,"Due in "&amp;F82-TODAY()&amp;IF(F82-TODAY()=1," day"," days"),"Next payment in "&amp;F82-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I82" s="1" t="n"/>
@@ -4602,7 +4618,7 @@
         <v/>
       </c>
       <c r="H83" s="33">
-        <f>IF(B83="","",IF(G83&lt;=0,"✓ Paid in full",IF(F83="","Balance, no date yet",IF(F83&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F83)&amp;" day(s)",IF(F83-TODAY()&lt;=14,"Due in "&amp;(F83-TODAY())&amp;" day(s)","Due "&amp;(F83-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B83="","",IF(G83&lt;=0,"Paid in full",IF(F83="","Balance due, no date set",IF(F83&lt;TODAY(),"Overdue by "&amp;TODAY()-F83&amp;IF(TODAY()-F83=1," day"," days"),IF(F83=TODAY(),"Due today",IF(F83-TODAY()&lt;=14,"Due in "&amp;F83-TODAY()&amp;IF(F83-TODAY()=1," day"," days"),"Next payment in "&amp;F83-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I83" s="1" t="n"/>
@@ -4619,7 +4635,7 @@
         <v/>
       </c>
       <c r="H84" s="33">
-        <f>IF(B84="","",IF(G84&lt;=0,"✓ Paid in full",IF(F84="","Balance, no date yet",IF(F84&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F84)&amp;" day(s)",IF(F84-TODAY()&lt;=14,"Due in "&amp;(F84-TODAY())&amp;" day(s)","Due "&amp;(F84-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B84="","",IF(G84&lt;=0,"Paid in full",IF(F84="","Balance due, no date set",IF(F84&lt;TODAY(),"Overdue by "&amp;TODAY()-F84&amp;IF(TODAY()-F84=1," day"," days"),IF(F84=TODAY(),"Due today",IF(F84-TODAY()&lt;=14,"Due in "&amp;F84-TODAY()&amp;IF(F84-TODAY()=1," day"," days"),"Next payment in "&amp;F84-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I84" s="1" t="n"/>
@@ -4636,7 +4652,7 @@
         <v/>
       </c>
       <c r="H85" s="33">
-        <f>IF(B85="","",IF(G85&lt;=0,"✓ Paid in full",IF(F85="","Balance, no date yet",IF(F85&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F85)&amp;" day(s)",IF(F85-TODAY()&lt;=14,"Due in "&amp;(F85-TODAY())&amp;" day(s)","Due "&amp;(F85-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B85="","",IF(G85&lt;=0,"Paid in full",IF(F85="","Balance due, no date set",IF(F85&lt;TODAY(),"Overdue by "&amp;TODAY()-F85&amp;IF(TODAY()-F85=1," day"," days"),IF(F85=TODAY(),"Due today",IF(F85-TODAY()&lt;=14,"Due in "&amp;F85-TODAY()&amp;IF(F85-TODAY()=1," day"," days"),"Next payment in "&amp;F85-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I85" s="1" t="n"/>
@@ -4653,7 +4669,7 @@
         <v/>
       </c>
       <c r="H86" s="33">
-        <f>IF(B86="","",IF(G86&lt;=0,"✓ Paid in full",IF(F86="","Balance, no date yet",IF(F86&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F86)&amp;" day(s)",IF(F86-TODAY()&lt;=14,"Due in "&amp;(F86-TODAY())&amp;" day(s)","Due "&amp;(F86-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B86="","",IF(G86&lt;=0,"Paid in full",IF(F86="","Balance due, no date set",IF(F86&lt;TODAY(),"Overdue by "&amp;TODAY()-F86&amp;IF(TODAY()-F86=1," day"," days"),IF(F86=TODAY(),"Due today",IF(F86-TODAY()&lt;=14,"Due in "&amp;F86-TODAY()&amp;IF(F86-TODAY()=1," day"," days"),"Next payment in "&amp;F86-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I86" s="1" t="n"/>
@@ -4670,7 +4686,7 @@
         <v/>
       </c>
       <c r="H87" s="33">
-        <f>IF(B87="","",IF(G87&lt;=0,"✓ Paid in full",IF(F87="","Balance, no date yet",IF(F87&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F87)&amp;" day(s)",IF(F87-TODAY()&lt;=14,"Due in "&amp;(F87-TODAY())&amp;" day(s)","Due "&amp;(F87-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B87="","",IF(G87&lt;=0,"Paid in full",IF(F87="","Balance due, no date set",IF(F87&lt;TODAY(),"Overdue by "&amp;TODAY()-F87&amp;IF(TODAY()-F87=1," day"," days"),IF(F87=TODAY(),"Due today",IF(F87-TODAY()&lt;=14,"Due in "&amp;F87-TODAY()&amp;IF(F87-TODAY()=1," day"," days"),"Next payment in "&amp;F87-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I87" s="1" t="n"/>
@@ -4687,7 +4703,7 @@
         <v/>
       </c>
       <c r="H88" s="33">
-        <f>IF(B88="","",IF(G88&lt;=0,"✓ Paid in full",IF(F88="","Balance, no date yet",IF(F88&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F88)&amp;" day(s)",IF(F88-TODAY()&lt;=14,"Due in "&amp;(F88-TODAY())&amp;" day(s)","Due "&amp;(F88-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B88="","",IF(G88&lt;=0,"Paid in full",IF(F88="","Balance due, no date set",IF(F88&lt;TODAY(),"Overdue by "&amp;TODAY()-F88&amp;IF(TODAY()-F88=1," day"," days"),IF(F88=TODAY(),"Due today",IF(F88-TODAY()&lt;=14,"Due in "&amp;F88-TODAY()&amp;IF(F88-TODAY()=1," day"," days"),"Next payment in "&amp;F88-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I88" s="1" t="n"/>
@@ -4704,7 +4720,7 @@
         <v/>
       </c>
       <c r="H89" s="33">
-        <f>IF(B89="","",IF(G89&lt;=0,"✓ Paid in full",IF(F89="","Balance, no date yet",IF(F89&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F89)&amp;" day(s)",IF(F89-TODAY()&lt;=14,"Due in "&amp;(F89-TODAY())&amp;" day(s)","Due "&amp;(F89-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B89="","",IF(G89&lt;=0,"Paid in full",IF(F89="","Balance due, no date set",IF(F89&lt;TODAY(),"Overdue by "&amp;TODAY()-F89&amp;IF(TODAY()-F89=1," day"," days"),IF(F89=TODAY(),"Due today",IF(F89-TODAY()&lt;=14,"Due in "&amp;F89-TODAY()&amp;IF(F89-TODAY()=1," day"," days"),"Next payment in "&amp;F89-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I89" s="1" t="n"/>
@@ -4721,7 +4737,7 @@
         <v/>
       </c>
       <c r="H90" s="33">
-        <f>IF(B90="","",IF(G90&lt;=0,"✓ Paid in full",IF(F90="","Balance, no date yet",IF(F90&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F90)&amp;" day(s)",IF(F90-TODAY()&lt;=14,"Due in "&amp;(F90-TODAY())&amp;" day(s)","Due "&amp;(F90-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B90="","",IF(G90&lt;=0,"Paid in full",IF(F90="","Balance due, no date set",IF(F90&lt;TODAY(),"Overdue by "&amp;TODAY()-F90&amp;IF(TODAY()-F90=1," day"," days"),IF(F90=TODAY(),"Due today",IF(F90-TODAY()&lt;=14,"Due in "&amp;F90-TODAY()&amp;IF(F90-TODAY()=1," day"," days"),"Next payment in "&amp;F90-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I90" s="1" t="n"/>
@@ -4738,7 +4754,7 @@
         <v/>
       </c>
       <c r="H91" s="33">
-        <f>IF(B91="","",IF(G91&lt;=0,"✓ Paid in full",IF(F91="","Balance, no date yet",IF(F91&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F91)&amp;" day(s)",IF(F91-TODAY()&lt;=14,"Due in "&amp;(F91-TODAY())&amp;" day(s)","Due "&amp;(F91-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B91="","",IF(G91&lt;=0,"Paid in full",IF(F91="","Balance due, no date set",IF(F91&lt;TODAY(),"Overdue by "&amp;TODAY()-F91&amp;IF(TODAY()-F91=1," day"," days"),IF(F91=TODAY(),"Due today",IF(F91-TODAY()&lt;=14,"Due in "&amp;F91-TODAY()&amp;IF(F91-TODAY()=1," day"," days"),"Next payment in "&amp;F91-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I91" s="1" t="n"/>
@@ -4755,7 +4771,7 @@
         <v/>
       </c>
       <c r="H92" s="33">
-        <f>IF(B92="","",IF(G92&lt;=0,"✓ Paid in full",IF(F92="","Balance, no date yet",IF(F92&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F92)&amp;" day(s)",IF(F92-TODAY()&lt;=14,"Due in "&amp;(F92-TODAY())&amp;" day(s)","Due "&amp;(F92-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B92="","",IF(G92&lt;=0,"Paid in full",IF(F92="","Balance due, no date set",IF(F92&lt;TODAY(),"Overdue by "&amp;TODAY()-F92&amp;IF(TODAY()-F92=1," day"," days"),IF(F92=TODAY(),"Due today",IF(F92-TODAY()&lt;=14,"Due in "&amp;F92-TODAY()&amp;IF(F92-TODAY()=1," day"," days"),"Next payment in "&amp;F92-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I92" s="1" t="n"/>
@@ -4772,7 +4788,7 @@
         <v/>
       </c>
       <c r="H93" s="33">
-        <f>IF(B93="","",IF(G93&lt;=0,"✓ Paid in full",IF(F93="","Balance, no date yet",IF(F93&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F93)&amp;" day(s)",IF(F93-TODAY()&lt;=14,"Due in "&amp;(F93-TODAY())&amp;" day(s)","Due "&amp;(F93-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B93="","",IF(G93&lt;=0,"Paid in full",IF(F93="","Balance due, no date set",IF(F93&lt;TODAY(),"Overdue by "&amp;TODAY()-F93&amp;IF(TODAY()-F93=1," day"," days"),IF(F93=TODAY(),"Due today",IF(F93-TODAY()&lt;=14,"Due in "&amp;F93-TODAY()&amp;IF(F93-TODAY()=1," day"," days"),"Next payment in "&amp;F93-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I93" s="1" t="n"/>
@@ -4789,7 +4805,7 @@
         <v/>
       </c>
       <c r="H94" s="33">
-        <f>IF(B94="","",IF(G94&lt;=0,"✓ Paid in full",IF(F94="","Balance, no date yet",IF(F94&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F94)&amp;" day(s)",IF(F94-TODAY()&lt;=14,"Due in "&amp;(F94-TODAY())&amp;" day(s)","Due "&amp;(F94-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B94="","",IF(G94&lt;=0,"Paid in full",IF(F94="","Balance due, no date set",IF(F94&lt;TODAY(),"Overdue by "&amp;TODAY()-F94&amp;IF(TODAY()-F94=1," day"," days"),IF(F94=TODAY(),"Due today",IF(F94-TODAY()&lt;=14,"Due in "&amp;F94-TODAY()&amp;IF(F94-TODAY()=1," day"," days"),"Next payment in "&amp;F94-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I94" s="1" t="n"/>
@@ -4806,7 +4822,7 @@
         <v/>
       </c>
       <c r="H95" s="33">
-        <f>IF(B95="","",IF(G95&lt;=0,"✓ Paid in full",IF(F95="","Balance, no date yet",IF(F95&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F95)&amp;" day(s)",IF(F95-TODAY()&lt;=14,"Due in "&amp;(F95-TODAY())&amp;" day(s)","Due "&amp;(F95-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B95="","",IF(G95&lt;=0,"Paid in full",IF(F95="","Balance due, no date set",IF(F95&lt;TODAY(),"Overdue by "&amp;TODAY()-F95&amp;IF(TODAY()-F95=1," day"," days"),IF(F95=TODAY(),"Due today",IF(F95-TODAY()&lt;=14,"Due in "&amp;F95-TODAY()&amp;IF(F95-TODAY()=1," day"," days"),"Next payment in "&amp;F95-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I95" s="1" t="n"/>
@@ -4823,7 +4839,7 @@
         <v/>
       </c>
       <c r="H96" s="33">
-        <f>IF(B96="","",IF(G96&lt;=0,"✓ Paid in full",IF(F96="","Balance, no date yet",IF(F96&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F96)&amp;" day(s)",IF(F96-TODAY()&lt;=14,"Due in "&amp;(F96-TODAY())&amp;" day(s)","Due "&amp;(F96-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B96="","",IF(G96&lt;=0,"Paid in full",IF(F96="","Balance due, no date set",IF(F96&lt;TODAY(),"Overdue by "&amp;TODAY()-F96&amp;IF(TODAY()-F96=1," day"," days"),IF(F96=TODAY(),"Due today",IF(F96-TODAY()&lt;=14,"Due in "&amp;F96-TODAY()&amp;IF(F96-TODAY()=1," day"," days"),"Next payment in "&amp;F96-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I96" s="1" t="n"/>
@@ -4840,7 +4856,7 @@
         <v/>
       </c>
       <c r="H97" s="33">
-        <f>IF(B97="","",IF(G97&lt;=0,"✓ Paid in full",IF(F97="","Balance, no date yet",IF(F97&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F97)&amp;" day(s)",IF(F97-TODAY()&lt;=14,"Due in "&amp;(F97-TODAY())&amp;" day(s)","Due "&amp;(F97-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B97="","",IF(G97&lt;=0,"Paid in full",IF(F97="","Balance due, no date set",IF(F97&lt;TODAY(),"Overdue by "&amp;TODAY()-F97&amp;IF(TODAY()-F97=1," day"," days"),IF(F97=TODAY(),"Due today",IF(F97-TODAY()&lt;=14,"Due in "&amp;F97-TODAY()&amp;IF(F97-TODAY()=1," day"," days"),"Next payment in "&amp;F97-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I97" s="1" t="n"/>
@@ -4857,7 +4873,7 @@
         <v/>
       </c>
       <c r="H98" s="33">
-        <f>IF(B98="","",IF(G98&lt;=0,"✓ Paid in full",IF(F98="","Balance, no date yet",IF(F98&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F98)&amp;" day(s)",IF(F98-TODAY()&lt;=14,"Due in "&amp;(F98-TODAY())&amp;" day(s)","Due "&amp;(F98-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B98="","",IF(G98&lt;=0,"Paid in full",IF(F98="","Balance due, no date set",IF(F98&lt;TODAY(),"Overdue by "&amp;TODAY()-F98&amp;IF(TODAY()-F98=1," day"," days"),IF(F98=TODAY(),"Due today",IF(F98-TODAY()&lt;=14,"Due in "&amp;F98-TODAY()&amp;IF(F98-TODAY()=1," day"," days"),"Next payment in "&amp;F98-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I98" s="1" t="n"/>
@@ -4874,7 +4890,7 @@
         <v/>
       </c>
       <c r="H99" s="33">
-        <f>IF(B99="","",IF(G99&lt;=0,"✓ Paid in full",IF(F99="","Balance, no date yet",IF(F99&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F99)&amp;" day(s)",IF(F99-TODAY()&lt;=14,"Due in "&amp;(F99-TODAY())&amp;" day(s)","Due "&amp;(F99-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B99="","",IF(G99&lt;=0,"Paid in full",IF(F99="","Balance due, no date set",IF(F99&lt;TODAY(),"Overdue by "&amp;TODAY()-F99&amp;IF(TODAY()-F99=1," day"," days"),IF(F99=TODAY(),"Due today",IF(F99-TODAY()&lt;=14,"Due in "&amp;F99-TODAY()&amp;IF(F99-TODAY()=1," day"," days"),"Next payment in "&amp;F99-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I99" s="1" t="n"/>
@@ -4891,7 +4907,7 @@
         <v/>
       </c>
       <c r="H100" s="33">
-        <f>IF(B100="","",IF(G100&lt;=0,"✓ Paid in full",IF(F100="","Balance, no date yet",IF(F100&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F100)&amp;" day(s)",IF(F100-TODAY()&lt;=14,"Due in "&amp;(F100-TODAY())&amp;" day(s)","Due "&amp;(F100-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B100="","",IF(G100&lt;=0,"Paid in full",IF(F100="","Balance due, no date set",IF(F100&lt;TODAY(),"Overdue by "&amp;TODAY()-F100&amp;IF(TODAY()-F100=1," day"," days"),IF(F100=TODAY(),"Due today",IF(F100-TODAY()&lt;=14,"Due in "&amp;F100-TODAY()&amp;IF(F100-TODAY()=1," day"," days"),"Next payment in "&amp;F100-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I100" s="1" t="n"/>
@@ -4908,7 +4924,7 @@
         <v/>
       </c>
       <c r="H101" s="33">
-        <f>IF(B101="","",IF(G101&lt;=0,"✓ Paid in full",IF(F101="","Balance, no date yet",IF(F101&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F101)&amp;" day(s)",IF(F101-TODAY()&lt;=14,"Due in "&amp;(F101-TODAY())&amp;" day(s)","Due "&amp;(F101-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B101="","",IF(G101&lt;=0,"Paid in full",IF(F101="","Balance due, no date set",IF(F101&lt;TODAY(),"Overdue by "&amp;TODAY()-F101&amp;IF(TODAY()-F101=1," day"," days"),IF(F101=TODAY(),"Due today",IF(F101-TODAY()&lt;=14,"Due in "&amp;F101-TODAY()&amp;IF(F101-TODAY()=1," day"," days"),"Next payment in "&amp;F101-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I101" s="1" t="n"/>
@@ -4925,7 +4941,7 @@
         <v/>
       </c>
       <c r="H102" s="33">
-        <f>IF(B102="","",IF(G102&lt;=0,"✓ Paid in full",IF(F102="","Balance, no date yet",IF(F102&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F102)&amp;" day(s)",IF(F102-TODAY()&lt;=14,"Due in "&amp;(F102-TODAY())&amp;" day(s)","Due "&amp;(F102-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B102="","",IF(G102&lt;=0,"Paid in full",IF(F102="","Balance due, no date set",IF(F102&lt;TODAY(),"Overdue by "&amp;TODAY()-F102&amp;IF(TODAY()-F102=1," day"," days"),IF(F102=TODAY(),"Due today",IF(F102-TODAY()&lt;=14,"Due in "&amp;F102-TODAY()&amp;IF(F102-TODAY()=1," day"," days"),"Next payment in "&amp;F102-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I102" s="1" t="n"/>
@@ -4942,7 +4958,7 @@
         <v/>
       </c>
       <c r="H103" s="33">
-        <f>IF(B103="","",IF(G103&lt;=0,"✓ Paid in full",IF(F103="","Balance, no date yet",IF(F103&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F103)&amp;" day(s)",IF(F103-TODAY()&lt;=14,"Due in "&amp;(F103-TODAY())&amp;" day(s)","Due "&amp;(F103-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B103="","",IF(G103&lt;=0,"Paid in full",IF(F103="","Balance due, no date set",IF(F103&lt;TODAY(),"Overdue by "&amp;TODAY()-F103&amp;IF(TODAY()-F103=1," day"," days"),IF(F103=TODAY(),"Due today",IF(F103-TODAY()&lt;=14,"Due in "&amp;F103-TODAY()&amp;IF(F103-TODAY()=1," day"," days"),"Next payment in "&amp;F103-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I103" s="1" t="n"/>
@@ -4959,7 +4975,7 @@
         <v/>
       </c>
       <c r="H104" s="33">
-        <f>IF(B104="","",IF(G104&lt;=0,"✓ Paid in full",IF(F104="","Balance, no date yet",IF(F104&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F104)&amp;" day(s)",IF(F104-TODAY()&lt;=14,"Due in "&amp;(F104-TODAY())&amp;" day(s)","Due "&amp;(F104-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B104="","",IF(G104&lt;=0,"Paid in full",IF(F104="","Balance due, no date set",IF(F104&lt;TODAY(),"Overdue by "&amp;TODAY()-F104&amp;IF(TODAY()-F104=1," day"," days"),IF(F104=TODAY(),"Due today",IF(F104-TODAY()&lt;=14,"Due in "&amp;F104-TODAY()&amp;IF(F104-TODAY()=1," day"," days"),"Next payment in "&amp;F104-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I104" s="1" t="n"/>
@@ -4976,7 +4992,7 @@
         <v/>
       </c>
       <c r="H105" s="33">
-        <f>IF(B105="","",IF(G105&lt;=0,"✓ Paid in full",IF(F105="","Balance, no date yet",IF(F105&lt;TODAY(),"⚠ OVERDUE "&amp;(TODAY()-F105)&amp;" day(s)",IF(F105-TODAY()&lt;=14,"Due in "&amp;(F105-TODAY())&amp;" day(s)","Due "&amp;(F105-TODAY())&amp;" days from now")))))</f>
+        <f>IF(B105="","",IF(G105&lt;=0,"Paid in full",IF(F105="","Balance due, no date set",IF(F105&lt;TODAY(),"Overdue by "&amp;TODAY()-F105&amp;IF(TODAY()-F105=1," day"," days"),IF(F105=TODAY(),"Due today",IF(F105-TODAY()&lt;=14,"Due in "&amp;F105-TODAY()&amp;IF(F105-TODAY()=1," day"," days"),"Next payment in "&amp;F105-TODAY()&amp;" days"))))))</f>
         <v/>
       </c>
       <c r="I105" s="1" t="n"/>
@@ -4994,14 +5010,14 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H6:H105">
-    <cfRule type="expression" priority="1" dxfId="2">
-      <formula>LEFT($H6,1)="✓"</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$H6="Paid in full"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>LEFT($H6,1)="⚠"</formula>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>LEFT($H6,7)="Overdue"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="3">
-      <formula>LEFT($H6,6)="Due in"</formula>
+      <formula>OR(LEFT($H6,6)="Due in",$H6="Due today")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -5141,8 +5157,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E6" s="34" t="b">
-        <v>1</v>
+      <c r="E6" s="34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="F6" s="34" t="inlineStr">
         <is>
@@ -5172,8 +5190,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E7" s="34" t="b">
-        <v>0</v>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
@@ -5203,8 +5223,10 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="E8" s="34" t="b">
-        <v>0</v>
+      <c r="E8" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F8" s="34" t="inlineStr"/>
       <c r="G8" s="25" t="n"/>
@@ -5228,8 +5250,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E9" s="34" t="b">
-        <v>0</v>
+      <c r="E9" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
@@ -5259,8 +5283,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E10" s="34" t="b">
-        <v>1</v>
+      <c r="E10" s="34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="F10" s="34" t="inlineStr"/>
       <c r="G10" s="25" t="n"/>
@@ -5284,8 +5310,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E11" s="34" t="b">
-        <v>0</v>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
@@ -5315,8 +5343,10 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="E12" s="34" t="b">
-        <v>0</v>
+      <c r="E12" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F12" s="34" t="inlineStr"/>
       <c r="G12" s="25" t="n"/>
@@ -5340,8 +5370,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E13" s="34" t="b">
-        <v>0</v>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
@@ -5371,8 +5403,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E14" s="34" t="b">
-        <v>1</v>
+      <c r="E14" s="34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="F14" s="34" t="inlineStr">
         <is>
@@ -5402,8 +5436,10 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="E15" s="34" t="b">
-        <v>0</v>
+      <c r="E15" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F15" s="34" t="inlineStr"/>
       <c r="G15" s="25" t="n"/>
@@ -5427,8 +5463,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E16" s="34" t="b">
-        <v>0</v>
+      <c r="E16" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
@@ -5458,8 +5496,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E17" s="34" t="b">
-        <v>0</v>
+      <c r="E17" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
@@ -8653,7 +8693,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D6:D305">
-    <cfRule type="expression" priority="1" dxfId="2">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D6="Yes"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="3">
@@ -8671,7 +8711,7 @@
       <formula1>"Yes,No,Pending"</formula1>
     </dataValidation>
     <dataValidation sqref="E6:E305" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="F6:F305" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Meat,Fish,Veggie,Kids"</formula1>
@@ -8706,7 +8746,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Start here: 10 minutes</t>
+          <t>Start here</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -8716,7 +8756,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Only type in YELLOW cells.</t>
+          <t>Type only in the yellow cells. Everything else is calculated.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -8737,7 +8777,7 @@
       </c>
       <c r="C5" s="36" t="inlineStr">
         <is>
-          <t>Dashboard: your wedding date (the countdown starts).</t>
+          <t>Dashboard: type your wedding date and the countdown starts.</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
@@ -8757,7 +8797,7 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>Budget: your total budget. Adjust the shares if your priorities differ (they must add up to 100).</t>
+          <t>Budget: type your total. Change the percentages if your priorities differ (they add up to 100).</t>
         </is>
       </c>
       <c r="D7" s="1" t="n"/>
@@ -8777,7 +8817,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Vendors: each vendor once you have a quote: amount, what you paid, next payment date.</t>
+          <t>Vendors: add each vendor once you have a quote, with the amount, what you paid and the next due date.</t>
         </is>
       </c>
       <c r="D9" s="1" t="n"/>
@@ -8797,7 +8837,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Guests: one line per guest; update RSVP and meal as answers come in.</t>
+          <t>Guests: one line per guest. Update the RSVP and meal as answers come in.</t>
         </is>
       </c>
       <c r="D11" s="1" t="n"/>
@@ -8812,12 +8852,12 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C13" s="36" t="inlineStr">
         <is>
-          <t>Dashboard: what is committed, paid and still to pay, payments due soon, and guest numbers.</t>
+          <t>The Dashboard then shows what is booked, paid and still to pay, and your guest numbers.</t>
         </is>
       </c>
       <c r="D13" s="1" t="n"/>
@@ -8845,7 +8885,7 @@
       <c r="B17" s="1" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Example vendors and guests show how it works: delete them and add yours.</t>
+          <t>The example vendors and guests show how it works. Delete them and add your own.</t>
         </is>
       </c>
       <c r="D17" s="1" t="n"/>
@@ -8861,7 +8901,7 @@
       <c r="B19" s="1" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Works in Google Sheets and Microsoft Excel. Any currency.</t>
+          <t>Works in Google Sheets and Microsoft Excel, in any currency.</t>
         </is>
       </c>
       <c r="D19" s="1" t="n"/>

</xml_diff>